<commit_message>
Sprint 6: reparto por historia completa entre Bryan, Catalina y Emilio
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/SIGMA_Pendientes_por_Sprint.xlsx
+++ b/Fase 2/Evidencias Proyecto/SIGMA_Pendientes_por_Sprint.xlsx
@@ -1119,7 +1119,7 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L7" s="8" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L9" s="8" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L17" s="8" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L19" s="8" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L24" s="8" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L25" s="8" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L26" s="8" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="K28" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L28" s="8" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L29" s="8" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L31" s="8" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L36" s="8" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="K37" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L37" s="8" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="K40" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L40" s="8" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L42" s="8" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L43" s="8" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="K44" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L44" s="8" t="inlineStr">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="K47" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L47" s="8" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="K48" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L48" s="8" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="K49" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L49" s="8" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="K50" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L50" s="8" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="K51" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L51" s="8" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="K52" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L52" s="8" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="K53" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L53" s="8" t="inlineStr">
@@ -4402,7 +4402,7 @@
       </c>
       <c r="K54" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L54" s="8" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="K55" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L55" s="8" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="K56" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L56" s="8" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="K57" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L57" s="8" t="inlineStr">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="K58" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L58" s="8" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="K59" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L59" s="8" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="K60" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L60" s="8" t="inlineStr">
@@ -4871,7 +4871,7 @@
       </c>
       <c r="K61" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L61" s="8" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="K62" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L62" s="8" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="K63" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L63" s="8" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="K64" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L64" s="8" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="K65" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L65" s="8" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="K66" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L66" s="8" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="K67" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L67" s="8" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="K68" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L68" s="8" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="K69" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L69" s="8" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="K70" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L70" s="8" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="K71" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L71" s="8" t="inlineStr">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="K72" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L72" s="8" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="K73" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L73" s="8" t="inlineStr">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="K74" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L74" s="8" t="inlineStr">
@@ -10834,7 +10834,7 @@
       </c>
       <c r="K150" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L150" s="8" t="inlineStr">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="K152" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L152" s="8" t="inlineStr">
@@ -11035,7 +11035,7 @@
       </c>
       <c r="K153" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L153" s="8" t="inlineStr">
@@ -11236,7 +11236,7 @@
       </c>
       <c r="K156" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L156" s="8" t="inlineStr">
@@ -11437,7 +11437,7 @@
       </c>
       <c r="K159" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L159" s="8" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="K160" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L160" s="8" t="inlineStr">
@@ -11571,7 +11571,7 @@
       </c>
       <c r="K161" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L161" s="8" t="inlineStr">
@@ -12442,7 +12442,7 @@
       </c>
       <c r="K174" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L174" s="8" t="inlineStr">
@@ -12509,7 +12509,7 @@
       </c>
       <c r="K175" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L175" s="8" t="inlineStr">
@@ -12576,7 +12576,7 @@
       </c>
       <c r="K176" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L176" s="8" t="inlineStr">
@@ -13380,7 +13380,7 @@
       </c>
       <c r="K188" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L188" s="8" t="inlineStr">
@@ -13447,7 +13447,7 @@
       </c>
       <c r="K189" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L189" s="8" t="inlineStr">
@@ -13514,7 +13514,7 @@
       </c>
       <c r="K190" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L190" s="8" t="inlineStr">
@@ -13581,7 +13581,7 @@
       </c>
       <c r="K191" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L191" s="8" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="K192" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L192" s="8" t="inlineStr">
@@ -13774,7 +13774,7 @@
       </c>
       <c r="K194" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L194" s="8" t="inlineStr">
@@ -13837,7 +13837,7 @@
       </c>
       <c r="K195" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L195" s="8" t="inlineStr">
@@ -13900,7 +13900,7 @@
       </c>
       <c r="K196" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L196" s="8" t="inlineStr">
@@ -13963,7 +13963,7 @@
       </c>
       <c r="K197" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L197" s="8" t="inlineStr">
@@ -14215,7 +14215,7 @@
       </c>
       <c r="K201" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L201" s="8" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="K206" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L206" s="8" t="inlineStr">
@@ -14751,7 +14751,7 @@
       </c>
       <c r="K209" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L209" s="8" t="inlineStr">
@@ -14818,7 +14818,7 @@
       </c>
       <c r="K210" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L210" s="8" t="inlineStr">
@@ -14885,7 +14885,7 @@
       </c>
       <c r="K211" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L211" s="8" t="inlineStr">
@@ -14952,7 +14952,7 @@
       </c>
       <c r="K212" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L212" s="8" t="inlineStr">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="K213" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L213" s="8" t="inlineStr">
@@ -15153,7 +15153,7 @@
       </c>
       <c r="K215" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L215" s="8" t="inlineStr">
@@ -15354,7 +15354,7 @@
       </c>
       <c r="K218" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L218" s="8" t="inlineStr">
@@ -15555,7 +15555,7 @@
       </c>
       <c r="K221" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L221" s="8" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="K222" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L222" s="8" t="inlineStr">
@@ -15689,7 +15689,7 @@
       </c>
       <c r="K223" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L223" s="8" t="inlineStr">
@@ -15823,7 +15823,7 @@
       </c>
       <c r="K225" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L225" s="8" t="inlineStr">
@@ -15890,7 +15890,7 @@
       </c>
       <c r="K226" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L226" s="8" t="inlineStr">
@@ -16091,7 +16091,7 @@
       </c>
       <c r="K229" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L229" s="8" t="inlineStr">
@@ -16292,7 +16292,7 @@
       </c>
       <c r="K232" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L232" s="8" t="inlineStr">
@@ -16493,7 +16493,7 @@
       </c>
       <c r="K235" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L235" s="8" t="inlineStr">
@@ -16560,7 +16560,7 @@
       </c>
       <c r="K236" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L236" s="8" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="K237" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L237" s="8" t="inlineStr">
@@ -16694,7 +16694,7 @@
       </c>
       <c r="K238" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L238" s="8" t="inlineStr">
@@ -16828,7 +16828,7 @@
       </c>
       <c r="K240" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L240" s="8" t="inlineStr">
@@ -16895,7 +16895,7 @@
       </c>
       <c r="K241" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L241" s="8" t="inlineStr">
@@ -17029,7 +17029,7 @@
       </c>
       <c r="K243" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L243" s="8" t="inlineStr">
@@ -17096,7 +17096,7 @@
       </c>
       <c r="K244" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L244" s="8" t="inlineStr">
@@ -17163,7 +17163,7 @@
       </c>
       <c r="K245" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L245" s="8" t="inlineStr">
@@ -17230,7 +17230,7 @@
       </c>
       <c r="K246" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L246" s="8" t="inlineStr">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="K251" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L251" s="8" t="inlineStr">
@@ -17632,7 +17632,7 @@
       </c>
       <c r="K252" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L252" s="8" t="inlineStr">
@@ -17766,7 +17766,7 @@
       </c>
       <c r="K254" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L254" s="8" t="inlineStr">
@@ -17900,7 +17900,7 @@
       </c>
       <c r="K256" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L256" s="8" t="inlineStr">
@@ -18034,7 +18034,7 @@
       </c>
       <c r="K258" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L258" s="8" t="inlineStr">
@@ -18235,7 +18235,7 @@
       </c>
       <c r="K261" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L261" s="8" t="inlineStr">
@@ -18302,7 +18302,7 @@
       </c>
       <c r="K262" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L262" s="8" t="inlineStr">
@@ -18369,7 +18369,7 @@
       </c>
       <c r="K263" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L263" s="8" t="inlineStr">
@@ -18436,7 +18436,7 @@
       </c>
       <c r="K264" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L264" s="8" t="inlineStr">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="K266" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L266" s="8" t="inlineStr">
@@ -18637,7 +18637,7 @@
       </c>
       <c r="K267" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L267" s="8" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="K268" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L268" s="8" t="inlineStr">
@@ -18771,7 +18771,7 @@
       </c>
       <c r="K269" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L269" s="8" t="inlineStr">
@@ -18838,7 +18838,7 @@
       </c>
       <c r="K270" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L270" s="8" t="inlineStr">
@@ -18905,7 +18905,7 @@
       </c>
       <c r="K271" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L271" s="8" t="inlineStr">
@@ -18972,7 +18972,7 @@
       </c>
       <c r="K272" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L272" s="8" t="inlineStr">
@@ -19039,7 +19039,7 @@
       </c>
       <c r="K273" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L273" s="8" t="inlineStr">
@@ -19307,7 +19307,7 @@
       </c>
       <c r="K277" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L277" s="8" t="inlineStr">
@@ -19374,7 +19374,7 @@
       </c>
       <c r="K278" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L278" s="8" t="inlineStr">
@@ -19508,7 +19508,7 @@
       </c>
       <c r="K280" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L280" s="8" t="inlineStr">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="K281" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L281" s="8" t="inlineStr">
@@ -19709,7 +19709,7 @@
       </c>
       <c r="K283" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L283" s="8" t="inlineStr">
@@ -19776,7 +19776,7 @@
       </c>
       <c r="K284" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L284" s="8" t="inlineStr">
@@ -19843,7 +19843,7 @@
       </c>
       <c r="K285" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L285" s="8" t="inlineStr">
@@ -19910,7 +19910,7 @@
       </c>
       <c r="K286" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L286" s="8" t="inlineStr">
@@ -20714,7 +20714,7 @@
       </c>
       <c r="K298" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L298" s="8" t="inlineStr">
@@ -20781,7 +20781,7 @@
       </c>
       <c r="K299" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L299" s="8" t="inlineStr">
@@ -20848,7 +20848,7 @@
       </c>
       <c r="K300" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L300" s="8" t="inlineStr">
@@ -20915,7 +20915,7 @@
       </c>
       <c r="K301" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L301" s="8" t="inlineStr">
@@ -20982,7 +20982,7 @@
       </c>
       <c r="K302" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L302" s="8" t="inlineStr">
@@ -21116,7 +21116,7 @@
       </c>
       <c r="K304" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L304" s="8" t="inlineStr">
@@ -21250,7 +21250,7 @@
       </c>
       <c r="K306" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L306" s="8" t="inlineStr">
@@ -21384,7 +21384,7 @@
       </c>
       <c r="K308" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L308" s="8" t="inlineStr">
@@ -21518,7 +21518,7 @@
       </c>
       <c r="K310" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L310" s="8" t="inlineStr">
@@ -21585,7 +21585,7 @@
       </c>
       <c r="K311" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L311" s="8" t="inlineStr">
@@ -21652,7 +21652,7 @@
       </c>
       <c r="K312" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L312" s="8" t="inlineStr">
@@ -21719,7 +21719,7 @@
       </c>
       <c r="K313" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L313" s="8" t="inlineStr">
@@ -21916,7 +21916,7 @@
       </c>
       <c r="K316" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L316" s="8" t="inlineStr">
@@ -21979,7 +21979,7 @@
       </c>
       <c r="K317" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L317" s="8" t="inlineStr">
@@ -22105,7 +22105,7 @@
       </c>
       <c r="K319" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L319" s="8" t="inlineStr">
@@ -22168,7 +22168,7 @@
       </c>
       <c r="K320" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L320" s="8" t="inlineStr">
@@ -22231,7 +22231,7 @@
       </c>
       <c r="K321" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L321" s="8" t="inlineStr">
@@ -22357,7 +22357,7 @@
       </c>
       <c r="K323" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L323" s="8" t="inlineStr">
@@ -22483,7 +22483,7 @@
       </c>
       <c r="K325" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L325" s="8" t="inlineStr">
@@ -22546,7 +22546,7 @@
       </c>
       <c r="K326" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L326" s="8" t="inlineStr">
@@ -22609,7 +22609,7 @@
       </c>
       <c r="K327" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L327" s="8" t="inlineStr">
@@ -22672,7 +22672,7 @@
       </c>
       <c r="K328" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L328" s="8" t="inlineStr">
@@ -22798,7 +22798,7 @@
       </c>
       <c r="K330" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L330" s="8" t="inlineStr">
@@ -22861,7 +22861,7 @@
       </c>
       <c r="K331" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L331" s="8" t="inlineStr">
@@ -22987,7 +22987,7 @@
       </c>
       <c r="K333" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L333" s="8" t="inlineStr">
@@ -23113,7 +23113,7 @@
       </c>
       <c r="K335" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L335" s="8" t="inlineStr">
@@ -23176,7 +23176,7 @@
       </c>
       <c r="K336" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L336" s="8" t="inlineStr">
@@ -23239,7 +23239,7 @@
       </c>
       <c r="K337" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L337" s="8" t="inlineStr">
@@ -23365,7 +23365,7 @@
       </c>
       <c r="K339" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L339" s="8" t="inlineStr">
@@ -23428,7 +23428,7 @@
       </c>
       <c r="K340" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L340" s="8" t="inlineStr">
@@ -23554,7 +23554,7 @@
       </c>
       <c r="K342" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L342" s="8" t="inlineStr">
@@ -23680,7 +23680,7 @@
       </c>
       <c r="K344" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L344" s="8" t="inlineStr">
@@ -23743,7 +23743,7 @@
       </c>
       <c r="K345" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L345" s="8" t="inlineStr">
@@ -23806,7 +23806,7 @@
       </c>
       <c r="K346" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L346" s="8" t="inlineStr">
@@ -23869,7 +23869,7 @@
       </c>
       <c r="K347" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L347" s="8" t="inlineStr">
@@ -23932,7 +23932,7 @@
       </c>
       <c r="K348" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L348" s="8" t="inlineStr">
@@ -23995,7 +23995,7 @@
       </c>
       <c r="K349" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L349" s="8" t="inlineStr">
@@ -24058,7 +24058,7 @@
       </c>
       <c r="K350" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L350" s="8" t="inlineStr">
@@ -24121,7 +24121,7 @@
       </c>
       <c r="K351" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L351" s="8" t="inlineStr">
@@ -24184,7 +24184,7 @@
       </c>
       <c r="K352" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L352" s="8" t="inlineStr">
@@ -24247,7 +24247,7 @@
       </c>
       <c r="K353" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L353" s="8" t="inlineStr">
@@ -24373,7 +24373,7 @@
       </c>
       <c r="K355" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L355" s="8" t="inlineStr">
@@ -24436,7 +24436,7 @@
       </c>
       <c r="K356" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L356" s="8" t="inlineStr">
@@ -24499,7 +24499,7 @@
       </c>
       <c r="K357" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L357" s="8" t="inlineStr">
@@ -24625,7 +24625,7 @@
       </c>
       <c r="K359" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L359" s="8" t="inlineStr">
@@ -24688,7 +24688,7 @@
       </c>
       <c r="K360" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L360" s="8" t="inlineStr">
@@ -24751,7 +24751,7 @@
       </c>
       <c r="K361" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L361" s="8" t="inlineStr">
@@ -24814,7 +24814,7 @@
       </c>
       <c r="K362" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L362" s="8" t="inlineStr">
@@ -24877,7 +24877,7 @@
       </c>
       <c r="K363" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L363" s="8" t="inlineStr">
@@ -24940,7 +24940,7 @@
       </c>
       <c r="K364" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L364" s="8" t="inlineStr">
@@ -25003,7 +25003,7 @@
       </c>
       <c r="K365" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L365" s="8" t="inlineStr">
@@ -25066,7 +25066,7 @@
       </c>
       <c r="K366" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L366" s="8" t="inlineStr">
@@ -25192,7 +25192,7 @@
       </c>
       <c r="K368" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L368" s="8" t="inlineStr">
@@ -25255,7 +25255,7 @@
       </c>
       <c r="K369" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L369" s="8" t="inlineStr">
@@ -25318,7 +25318,7 @@
       </c>
       <c r="K370" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L370" s="8" t="inlineStr">
@@ -25444,7 +25444,7 @@
       </c>
       <c r="K372" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L372" s="8" t="inlineStr">
@@ -25507,7 +25507,7 @@
       </c>
       <c r="K373" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L373" s="8" t="inlineStr">
@@ -25570,7 +25570,7 @@
       </c>
       <c r="K374" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L374" s="8" t="inlineStr">
@@ -25633,7 +25633,7 @@
       </c>
       <c r="K375" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L375" s="8" t="inlineStr">
@@ -25696,7 +25696,7 @@
       </c>
       <c r="K376" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L376" s="8" t="inlineStr">
@@ -25759,7 +25759,7 @@
       </c>
       <c r="K377" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L377" s="8" t="inlineStr">
@@ -25822,7 +25822,7 @@
       </c>
       <c r="K378" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L378" s="8" t="inlineStr">
@@ -25948,7 +25948,7 @@
       </c>
       <c r="K380" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L380" s="8" t="inlineStr">
@@ -26011,7 +26011,7 @@
       </c>
       <c r="K381" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L381" s="8" t="inlineStr">
@@ -26074,7 +26074,7 @@
       </c>
       <c r="K382" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L382" s="8" t="inlineStr">
@@ -26200,7 +26200,7 @@
       </c>
       <c r="K384" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L384" s="8" t="inlineStr">
@@ -26326,7 +26326,7 @@
       </c>
       <c r="K386" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L386" s="8" t="inlineStr">
@@ -26389,7 +26389,7 @@
       </c>
       <c r="K387" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L387" s="8" t="inlineStr">
@@ -26452,7 +26452,7 @@
       </c>
       <c r="K388" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L388" s="8" t="inlineStr">
@@ -26578,7 +26578,7 @@
       </c>
       <c r="K390" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L390" s="8" t="inlineStr">
@@ -26641,7 +26641,7 @@
       </c>
       <c r="K391" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L391" s="8" t="inlineStr">
@@ -26767,7 +26767,7 @@
       </c>
       <c r="K393" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L393" s="8" t="inlineStr">
@@ -26956,7 +26956,7 @@
       </c>
       <c r="K396" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L396" s="8" t="inlineStr">
@@ -27019,7 +27019,7 @@
       </c>
       <c r="K397" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L397" s="8" t="inlineStr">
@@ -27082,7 +27082,7 @@
       </c>
       <c r="K398" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L398" s="8" t="inlineStr">
@@ -27145,7 +27145,7 @@
       </c>
       <c r="K399" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L399" s="8" t="inlineStr">
@@ -27271,7 +27271,7 @@
       </c>
       <c r="K401" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L401" s="8" t="inlineStr">
@@ -27397,7 +27397,7 @@
       </c>
       <c r="K403" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L403" s="8" t="inlineStr">
@@ -27460,7 +27460,7 @@
       </c>
       <c r="K404" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L404" s="8" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="K405" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L405" s="8" t="inlineStr">
@@ -27586,7 +27586,7 @@
       </c>
       <c r="K406" s="8" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="L406" s="8" t="inlineStr">
@@ -27649,7 +27649,7 @@
       </c>
       <c r="K407" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L407" s="8" t="inlineStr">
@@ -27712,7 +27712,7 @@
       </c>
       <c r="K408" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L408" s="8" t="inlineStr">
@@ -27838,7 +27838,7 @@
       </c>
       <c r="K410" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L410" s="8" t="inlineStr">
@@ -27901,7 +27901,7 @@
       </c>
       <c r="K411" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L411" s="8" t="inlineStr">
@@ -27964,7 +27964,7 @@
       </c>
       <c r="K412" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L412" s="8" t="inlineStr">
@@ -28216,7 +28216,7 @@
       </c>
       <c r="K416" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L416" s="8" t="inlineStr">
@@ -28279,7 +28279,7 @@
       </c>
       <c r="K417" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L417" s="8" t="inlineStr">
@@ -28405,7 +28405,7 @@
       </c>
       <c r="K419" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L419" s="8" t="inlineStr">
@@ -28468,7 +28468,7 @@
       </c>
       <c r="K420" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L420" s="8" t="inlineStr">
@@ -28531,7 +28531,7 @@
       </c>
       <c r="K421" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L421" s="8" t="inlineStr">
@@ -28594,7 +28594,7 @@
       </c>
       <c r="K422" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L422" s="8" t="inlineStr">
@@ -28657,7 +28657,7 @@
       </c>
       <c r="K423" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L423" s="8" t="inlineStr">
@@ -28909,7 +28909,7 @@
       </c>
       <c r="K427" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L427" s="8" t="inlineStr">
@@ -28972,7 +28972,7 @@
       </c>
       <c r="K428" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L428" s="8" t="inlineStr">
@@ -29098,7 +29098,7 @@
       </c>
       <c r="K430" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L430" s="8" t="inlineStr">
@@ -29161,7 +29161,7 @@
       </c>
       <c r="K431" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L431" s="8" t="inlineStr">
@@ -29224,7 +29224,7 @@
       </c>
       <c r="K432" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L432" s="8" t="inlineStr">
@@ -29413,7 +29413,7 @@
       </c>
       <c r="K435" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="L435" s="8" t="inlineStr">
@@ -29480,7 +29480,7 @@
       </c>
       <c r="K436" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L436" s="8" t="inlineStr">
@@ -29543,7 +29543,7 @@
       </c>
       <c r="K437" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L437" s="8" t="inlineStr">
@@ -29669,7 +29669,7 @@
       </c>
       <c r="K439" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L439" s="8" t="inlineStr">
@@ -29732,7 +29732,7 @@
       </c>
       <c r="K440" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L440" s="8" t="inlineStr">
@@ -29795,7 +29795,7 @@
       </c>
       <c r="K441" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L441" s="8" t="inlineStr">
@@ -29858,7 +29858,7 @@
       </c>
       <c r="K442" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L442" s="8" t="inlineStr">
@@ -30173,7 +30173,7 @@
       </c>
       <c r="K447" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L447" s="8" t="inlineStr">
@@ -30236,7 +30236,7 @@
       </c>
       <c r="K448" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L448" s="8" t="inlineStr">
@@ -30362,7 +30362,7 @@
       </c>
       <c r="K450" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L450" s="8" t="inlineStr">
@@ -30425,7 +30425,7 @@
       </c>
       <c r="K451" s="8" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L451" s="8" t="inlineStr">
@@ -30488,7 +30488,7 @@
       </c>
       <c r="K452" s="8" t="inlineStr">
         <is>
-          <t>Bryan Chávez</t>
+          <t>Catalina Pescio</t>
         </is>
       </c>
       <c r="L452" s="8" t="inlineStr">
@@ -30782,7 +30782,7 @@
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="5" t="n">
-        <v>172.8</v>
+        <v>117.8</v>
       </c>
       <c r="I6" s="6">
         <f>SUM(C6:H6)</f>
@@ -30801,7 +30801,7 @@
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="n">
-        <v>82.2</v>
+        <v>117</v>
       </c>
       <c r="I7" s="6">
         <f>SUM(C7:H7)</f>
@@ -30820,7 +30820,7 @@
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="5" t="n">
-        <v>98.2</v>
+        <v>118.5</v>
       </c>
       <c r="I8" s="6">
         <f>SUM(C8:H8)</f>

</xml_diff>